<commit_message>
Pushing daily stats for March 25, 2026
</commit_message>
<xml_diff>
--- a/assets/Combined_Daily_Data.xlsx
+++ b/assets/Combined_Daily_Data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="70">
   <si>
     <t>fg_name</t>
   </si>
@@ -172,9 +172,6 @@
     <t>Aaron Judge</t>
   </si>
   <si>
-    <t>Anthony Volpe</t>
-  </si>
-  <si>
     <t>Austin Wells</t>
   </si>
   <si>
@@ -226,7 +223,7 @@
     <t>vs L</t>
   </si>
   <si>
-    <t>March 24</t>
+    <t>March 25</t>
   </si>
 </sst>
 </file>
@@ -584,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AY10"/>
+  <dimension ref="A1:AY9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:51">
@@ -747,10 +744,10 @@
         <v>51</v>
       </c>
       <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" t="s">
         <v>60</v>
-      </c>
-      <c r="C2" t="s">
-        <v>61</v>
       </c>
       <c r="D2" t="s">
         <v>51</v>
@@ -759,10 +756,10 @@
         <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H2">
         <v>2</v>
@@ -813,22 +810,22 @@
         <v>44.5</v>
       </c>
       <c r="X2" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y2" t="s">
         <v>66</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" t="s">
-        <v>68</v>
-      </c>
       <c r="AA2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AB2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AC2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AD2">
         <v>428</v>
@@ -894,7 +891,7 @@
         <v>1</v>
       </c>
       <c r="AY2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:51">
@@ -902,10 +899,10 @@
         <v>52</v>
       </c>
       <c r="B3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" t="s">
         <v>60</v>
-      </c>
-      <c r="C3" t="s">
-        <v>61</v>
       </c>
       <c r="D3" t="s">
         <v>52</v>
@@ -917,115 +914,115 @@
         <v>63</v>
       </c>
       <c r="G3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>385</v>
+        <v>276</v>
       </c>
       <c r="J3">
         <v>15</v>
       </c>
       <c r="K3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>0.195</v>
+        <v>0.21</v>
       </c>
       <c r="N3">
-        <v>0.274</v>
+        <v>0.298</v>
       </c>
       <c r="O3">
-        <v>0.187</v>
+        <v>0.221</v>
       </c>
       <c r="P3">
-        <v>0.254</v>
+        <v>0.271</v>
       </c>
       <c r="Q3">
-        <v>0.382</v>
+        <v>0.431</v>
       </c>
       <c r="R3">
-        <v>0.635</v>
+        <v>0.702</v>
       </c>
       <c r="S3">
-        <v>25.7</v>
+        <v>26.7</v>
       </c>
       <c r="T3">
-        <v>6.8</v>
+        <v>7.1</v>
       </c>
       <c r="U3">
-        <v>39.3</v>
+        <v>30.3</v>
       </c>
       <c r="V3">
-        <v>46.1</v>
+        <v>52.7</v>
       </c>
       <c r="W3">
-        <v>32.2</v>
+        <v>34.3</v>
       </c>
       <c r="X3" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y3" t="s">
         <v>66</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>67</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC3" t="s">
         <v>68</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>65</v>
       </c>
       <c r="AD3">
         <v>428</v>
       </c>
       <c r="AE3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AF3">
-        <v>0.242</v>
+        <v>0.286</v>
       </c>
       <c r="AG3">
-        <v>0.274</v>
+        <v>0.332</v>
       </c>
       <c r="AH3">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="AI3">
-        <v>0.08600000000000002</v>
+        <v>0.158</v>
       </c>
       <c r="AJ3">
-        <v>0.328</v>
+        <v>0.444</v>
       </c>
       <c r="AK3">
-        <v>28</v>
+        <v>24.3</v>
       </c>
       <c r="AL3">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="AM3">
-        <v>2.4</v>
+        <v>2.82</v>
       </c>
       <c r="AN3">
-        <v>53</v>
+        <v>53.4</v>
       </c>
       <c r="AO3">
-        <v>25.4</v>
+        <v>24.3</v>
       </c>
       <c r="AP3">
-        <v>8.5</v>
+        <v>11.3</v>
       </c>
       <c r="AQ3">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="AR3">
         <v>1</v>
@@ -1040,7 +1037,7 @@
         <v>1</v>
       </c>
       <c r="AV3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW3">
         <v>0</v>
@@ -1049,7 +1046,7 @@
         <v>0</v>
       </c>
       <c r="AY3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:51">
@@ -1057,10 +1054,10 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
@@ -1069,76 +1066,76 @@
         <v>53</v>
       </c>
       <c r="F4" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" t="s">
         <v>64</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>361</v>
+      </c>
+      <c r="J4">
+        <v>19</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>0.269</v>
+      </c>
+      <c r="N4">
+        <v>0.371</v>
+      </c>
+      <c r="O4">
+        <v>0.235</v>
+      </c>
+      <c r="P4">
+        <v>0.356</v>
+      </c>
+      <c r="Q4">
+        <v>0.504</v>
+      </c>
+      <c r="R4">
+        <v>0.86</v>
+      </c>
+      <c r="S4">
+        <v>16.3</v>
+      </c>
+      <c r="T4">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="U4">
+        <v>39.1</v>
+      </c>
+      <c r="V4">
+        <v>40.8</v>
+      </c>
+      <c r="W4">
+        <v>42.9</v>
+      </c>
+      <c r="X4" t="s">
         <v>65</v>
       </c>
-      <c r="H4">
-        <v>7</v>
-      </c>
-      <c r="I4">
-        <v>276</v>
-      </c>
-      <c r="J4">
-        <v>15</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>0.21</v>
-      </c>
-      <c r="N4">
-        <v>0.298</v>
-      </c>
-      <c r="O4">
-        <v>0.221</v>
-      </c>
-      <c r="P4">
-        <v>0.271</v>
-      </c>
-      <c r="Q4">
-        <v>0.431</v>
-      </c>
-      <c r="R4">
-        <v>0.702</v>
-      </c>
-      <c r="S4">
-        <v>26.7</v>
-      </c>
-      <c r="T4">
-        <v>7.1</v>
-      </c>
-      <c r="U4">
-        <v>30.3</v>
-      </c>
-      <c r="V4">
-        <v>52.7</v>
-      </c>
-      <c r="W4">
-        <v>34.3</v>
-      </c>
-      <c r="X4" t="s">
+      <c r="Y4" t="s">
         <v>66</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>67</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC4" t="s">
         <v>68</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>69</v>
       </c>
       <c r="AD4">
         <v>428</v>
@@ -1183,16 +1180,16 @@
         <v>27.4</v>
       </c>
       <c r="AR4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT4">
         <v>0</v>
       </c>
       <c r="AU4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV4">
         <v>1</v>
@@ -1201,10 +1198,10 @@
         <v>0</v>
       </c>
       <c r="AX4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:51">
@@ -1212,10 +1209,10 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" t="s">
         <v>60</v>
-      </c>
-      <c r="C5" t="s">
-        <v>61</v>
       </c>
       <c r="D5" t="s">
         <v>54</v>
@@ -1224,76 +1221,76 @@
         <v>54</v>
       </c>
       <c r="F5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" t="s">
         <v>64</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>435</v>
+      </c>
+      <c r="J5">
+        <v>21</v>
+      </c>
+      <c r="K5">
+        <v>8</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0.244</v>
+      </c>
+      <c r="N5">
+        <v>0.318</v>
+      </c>
+      <c r="O5">
+        <v>0.193</v>
+      </c>
+      <c r="P5">
+        <v>0.304</v>
+      </c>
+      <c r="Q5">
+        <v>0.437</v>
+      </c>
+      <c r="R5">
+        <v>0.741</v>
+      </c>
+      <c r="S5">
+        <v>15.2</v>
+      </c>
+      <c r="T5">
+        <v>8.1</v>
+      </c>
+      <c r="U5">
+        <v>32.2</v>
+      </c>
+      <c r="V5">
+        <v>47.8</v>
+      </c>
+      <c r="W5">
+        <v>27.7</v>
+      </c>
+      <c r="X5" t="s">
         <v>65</v>
       </c>
-      <c r="H5">
-        <v>3</v>
-      </c>
-      <c r="I5">
-        <v>361</v>
-      </c>
-      <c r="J5">
-        <v>19</v>
-      </c>
-      <c r="K5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>0.269</v>
-      </c>
-      <c r="N5">
-        <v>0.371</v>
-      </c>
-      <c r="O5">
-        <v>0.235</v>
-      </c>
-      <c r="P5">
-        <v>0.356</v>
-      </c>
-      <c r="Q5">
-        <v>0.504</v>
-      </c>
-      <c r="R5">
-        <v>0.86</v>
-      </c>
-      <c r="S5">
-        <v>16.3</v>
-      </c>
-      <c r="T5">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="U5">
-        <v>39.1</v>
-      </c>
-      <c r="V5">
-        <v>40.8</v>
-      </c>
-      <c r="W5">
-        <v>42.9</v>
-      </c>
-      <c r="X5" t="s">
+      <c r="Y5" t="s">
         <v>66</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>67</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC5" t="s">
         <v>68</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>69</v>
       </c>
       <c r="AD5">
         <v>428</v>
@@ -1341,7 +1338,7 @@
         <v>0</v>
       </c>
       <c r="AS5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT5">
         <v>0</v>
@@ -1350,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="AV5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW5">
         <v>0</v>
       </c>
       <c r="AX5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:51">
@@ -1367,10 +1364,10 @@
         <v>55</v>
       </c>
       <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
         <v>60</v>
-      </c>
-      <c r="C6" t="s">
-        <v>61</v>
       </c>
       <c r="D6" t="s">
         <v>55</v>
@@ -1379,142 +1376,142 @@
         <v>55</v>
       </c>
       <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" t="s">
         <v>64</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>184</v>
+      </c>
+      <c r="J6">
+        <v>19</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0.272</v>
+      </c>
+      <c r="N6">
+        <v>0.395</v>
+      </c>
+      <c r="O6">
+        <v>0.337</v>
+      </c>
+      <c r="P6">
+        <v>0.332</v>
+      </c>
+      <c r="Q6">
+        <v>0.609</v>
+      </c>
+      <c r="R6">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="S6">
+        <v>35.5</v>
+      </c>
+      <c r="T6">
+        <v>7.9</v>
+      </c>
+      <c r="U6">
+        <v>32.7</v>
+      </c>
+      <c r="V6">
+        <v>44.2</v>
+      </c>
+      <c r="W6">
+        <v>46.9</v>
+      </c>
+      <c r="X6" t="s">
         <v>65</v>
       </c>
-      <c r="H6">
-        <v>4</v>
-      </c>
-      <c r="I6">
-        <v>435</v>
-      </c>
-      <c r="J6">
-        <v>21</v>
-      </c>
-      <c r="K6">
-        <v>8</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0.244</v>
-      </c>
-      <c r="N6">
-        <v>0.318</v>
-      </c>
-      <c r="O6">
-        <v>0.193</v>
-      </c>
-      <c r="P6">
-        <v>0.304</v>
-      </c>
-      <c r="Q6">
-        <v>0.437</v>
-      </c>
-      <c r="R6">
-        <v>0.741</v>
-      </c>
-      <c r="S6">
-        <v>15.2</v>
-      </c>
-      <c r="T6">
-        <v>8.1</v>
-      </c>
-      <c r="U6">
-        <v>32.2</v>
-      </c>
-      <c r="V6">
-        <v>47.8</v>
-      </c>
-      <c r="W6">
-        <v>27.7</v>
-      </c>
-      <c r="X6" t="s">
+      <c r="Y6" t="s">
         <v>66</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>67</v>
       </c>
-      <c r="Z6" t="s">
-        <v>68</v>
-      </c>
       <c r="AA6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AB6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AC6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="AD6">
         <v>428</v>
       </c>
       <c r="AE6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AF6">
-        <v>0.286</v>
+        <v>0.242</v>
       </c>
       <c r="AG6">
-        <v>0.332</v>
+        <v>0.274</v>
       </c>
       <c r="AH6">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="AI6">
-        <v>0.158</v>
+        <v>0.08600000000000002</v>
       </c>
       <c r="AJ6">
-        <v>0.444</v>
+        <v>0.328</v>
       </c>
       <c r="AK6">
-        <v>24.3</v>
+        <v>28</v>
       </c>
       <c r="AL6">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="AM6">
-        <v>2.82</v>
+        <v>2.4</v>
       </c>
       <c r="AN6">
-        <v>53.4</v>
+        <v>53</v>
       </c>
       <c r="AO6">
-        <v>24.3</v>
+        <v>25.4</v>
       </c>
       <c r="AP6">
-        <v>11.3</v>
+        <v>8.5</v>
       </c>
       <c r="AQ6">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="AR6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS6">
         <v>0</v>
       </c>
       <c r="AT6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU6">
         <v>0</v>
       </c>
       <c r="AV6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW6">
         <v>0</v>
       </c>
       <c r="AX6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:51">
@@ -1522,139 +1519,139 @@
         <v>56</v>
       </c>
       <c r="B7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" t="s">
         <v>60</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" t="s">
-        <v>56</v>
-      </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F7" t="s">
         <v>63</v>
       </c>
       <c r="G7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+      <c r="I7">
+        <v>333</v>
+      </c>
+      <c r="J7">
+        <v>25</v>
+      </c>
+      <c r="K7">
+        <v>28</v>
+      </c>
+      <c r="L7">
+        <v>5</v>
+      </c>
+      <c r="M7">
+        <v>0.24</v>
+      </c>
+      <c r="N7">
+        <v>0.36</v>
+      </c>
+      <c r="O7">
+        <v>0.267</v>
+      </c>
+      <c r="P7">
+        <v>0.336</v>
+      </c>
+      <c r="Q7">
+        <v>0.508</v>
+      </c>
+      <c r="R7">
+        <v>0.843</v>
+      </c>
+      <c r="S7">
+        <v>29.2</v>
+      </c>
+      <c r="T7">
+        <v>12.2</v>
+      </c>
+      <c r="U7">
+        <v>34.7</v>
+      </c>
+      <c r="V7">
+        <v>49.5</v>
+      </c>
+      <c r="W7">
+        <v>33.6</v>
+      </c>
+      <c r="X7" t="s">
         <v>65</v>
       </c>
-      <c r="H7">
-        <v>5</v>
-      </c>
-      <c r="I7">
-        <v>184</v>
-      </c>
-      <c r="J7">
-        <v>19</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0.272</v>
-      </c>
-      <c r="N7">
-        <v>0.395</v>
-      </c>
-      <c r="O7">
-        <v>0.337</v>
-      </c>
-      <c r="P7">
-        <v>0.332</v>
-      </c>
-      <c r="Q7">
-        <v>0.609</v>
-      </c>
-      <c r="R7">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="S7">
-        <v>35.5</v>
-      </c>
-      <c r="T7">
-        <v>7.9</v>
-      </c>
-      <c r="U7">
-        <v>32.7</v>
-      </c>
-      <c r="V7">
-        <v>44.2</v>
-      </c>
-      <c r="W7">
-        <v>46.9</v>
-      </c>
-      <c r="X7" t="s">
+      <c r="Y7" t="s">
         <v>66</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>67</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC7" t="s">
         <v>68</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>65</v>
       </c>
       <c r="AD7">
         <v>428</v>
       </c>
       <c r="AE7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AF7">
-        <v>0.242</v>
+        <v>0.286</v>
       </c>
       <c r="AG7">
-        <v>0.274</v>
+        <v>0.332</v>
       </c>
       <c r="AH7">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="AI7">
-        <v>0.08600000000000002</v>
+        <v>0.158</v>
       </c>
       <c r="AJ7">
-        <v>0.328</v>
+        <v>0.444</v>
       </c>
       <c r="AK7">
-        <v>28</v>
+        <v>24.3</v>
       </c>
       <c r="AL7">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="AM7">
-        <v>2.4</v>
+        <v>2.82</v>
       </c>
       <c r="AN7">
-        <v>53</v>
+        <v>53.4</v>
       </c>
       <c r="AO7">
-        <v>25.4</v>
+        <v>24.3</v>
       </c>
       <c r="AP7">
-        <v>8.5</v>
+        <v>11.3</v>
       </c>
       <c r="AQ7">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="AR7">
         <v>1</v>
       </c>
       <c r="AS7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU7">
         <v>0</v>
@@ -1666,10 +1663,10 @@
         <v>0</v>
       </c>
       <c r="AX7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:51">
@@ -1677,88 +1674,88 @@
         <v>57</v>
       </c>
       <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" t="s">
         <v>60</v>
       </c>
-      <c r="C8" t="s">
-        <v>61</v>
-      </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
         <v>64</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8">
+        <v>9</v>
+      </c>
+      <c r="I8">
+        <v>395</v>
+      </c>
+      <c r="J8">
+        <v>18</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>0.223</v>
+      </c>
+      <c r="N8">
+        <v>0.323</v>
+      </c>
+      <c r="O8">
+        <v>0.192</v>
+      </c>
+      <c r="P8">
+        <v>0.324</v>
+      </c>
+      <c r="Q8">
+        <v>0.415</v>
+      </c>
+      <c r="R8">
+        <v>0.739</v>
+      </c>
+      <c r="S8">
+        <v>32.4</v>
+      </c>
+      <c r="T8">
+        <v>12.7</v>
+      </c>
+      <c r="U8">
+        <v>40.3</v>
+      </c>
+      <c r="V8">
+        <v>40.3</v>
+      </c>
+      <c r="W8">
+        <v>40</v>
+      </c>
+      <c r="X8" t="s">
         <v>65</v>
       </c>
-      <c r="H8">
-        <v>6</v>
-      </c>
-      <c r="I8">
-        <v>333</v>
-      </c>
-      <c r="J8">
-        <v>25</v>
-      </c>
-      <c r="K8">
-        <v>28</v>
-      </c>
-      <c r="L8">
-        <v>5</v>
-      </c>
-      <c r="M8">
-        <v>0.24</v>
-      </c>
-      <c r="N8">
-        <v>0.36</v>
-      </c>
-      <c r="O8">
-        <v>0.267</v>
-      </c>
-      <c r="P8">
-        <v>0.336</v>
-      </c>
-      <c r="Q8">
-        <v>0.508</v>
-      </c>
-      <c r="R8">
-        <v>0.843</v>
-      </c>
-      <c r="S8">
-        <v>29.2</v>
-      </c>
-      <c r="T8">
-        <v>12.2</v>
-      </c>
-      <c r="U8">
-        <v>34.7</v>
-      </c>
-      <c r="V8">
-        <v>49.5</v>
-      </c>
-      <c r="W8">
-        <v>33.6</v>
-      </c>
-      <c r="X8" t="s">
+      <c r="Y8" t="s">
         <v>66</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Z8" t="s">
         <v>67</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC8" t="s">
         <v>68</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC8" t="s">
-        <v>69</v>
       </c>
       <c r="AD8">
         <v>428</v>
@@ -1812,19 +1809,19 @@
         <v>0</v>
       </c>
       <c r="AU8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW8">
         <v>0</v>
       </c>
       <c r="AX8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:51">
@@ -1832,10 +1829,10 @@
         <v>58</v>
       </c>
       <c r="B9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" t="s">
         <v>60</v>
-      </c>
-      <c r="C9" t="s">
-        <v>61</v>
       </c>
       <c r="D9" t="s">
         <v>58</v>
@@ -1844,76 +1841,76 @@
         <v>58</v>
       </c>
       <c r="F9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" t="s">
         <v>64</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>362</v>
+      </c>
+      <c r="J9">
+        <v>27</v>
+      </c>
+      <c r="K9">
+        <v>3</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>0.254</v>
+      </c>
+      <c r="N9">
+        <v>0.375</v>
+      </c>
+      <c r="O9">
+        <v>0.251</v>
+      </c>
+      <c r="P9">
+        <v>0.364</v>
+      </c>
+      <c r="Q9">
+        <v>0.506</v>
+      </c>
+      <c r="R9">
+        <v>0.869</v>
+      </c>
+      <c r="S9">
+        <v>22.5</v>
+      </c>
+      <c r="T9">
+        <v>14.3</v>
+      </c>
+      <c r="U9">
+        <v>33.2</v>
+      </c>
+      <c r="V9">
+        <v>48.7</v>
+      </c>
+      <c r="W9">
+        <v>37.5</v>
+      </c>
+      <c r="X9" t="s">
         <v>65</v>
       </c>
-      <c r="H9">
-        <v>9</v>
-      </c>
-      <c r="I9">
-        <v>395</v>
-      </c>
-      <c r="J9">
-        <v>18</v>
-      </c>
-      <c r="K9">
-        <v>2</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9">
-        <v>0.223</v>
-      </c>
-      <c r="N9">
-        <v>0.323</v>
-      </c>
-      <c r="O9">
-        <v>0.192</v>
-      </c>
-      <c r="P9">
-        <v>0.324</v>
-      </c>
-      <c r="Q9">
-        <v>0.415</v>
-      </c>
-      <c r="R9">
-        <v>0.739</v>
-      </c>
-      <c r="S9">
-        <v>32.4</v>
-      </c>
-      <c r="T9">
-        <v>12.7</v>
-      </c>
-      <c r="U9">
-        <v>40.3</v>
-      </c>
-      <c r="V9">
-        <v>40.3</v>
-      </c>
-      <c r="W9">
-        <v>40</v>
-      </c>
-      <c r="X9" t="s">
+      <c r="Y9" t="s">
         <v>66</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z9" t="s">
         <v>67</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC9" t="s">
         <v>68</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>69</v>
       </c>
       <c r="AD9">
         <v>428</v>
@@ -1967,10 +1964,10 @@
         <v>0</v>
       </c>
       <c r="AU9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW9">
         <v>0</v>
@@ -1979,162 +1976,7 @@
         <v>1</v>
       </c>
       <c r="AY9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:51">
-      <c r="A10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>362</v>
-      </c>
-      <c r="J10">
-        <v>27</v>
-      </c>
-      <c r="K10">
-        <v>3</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10">
-        <v>0.254</v>
-      </c>
-      <c r="N10">
-        <v>0.375</v>
-      </c>
-      <c r="O10">
-        <v>0.251</v>
-      </c>
-      <c r="P10">
-        <v>0.364</v>
-      </c>
-      <c r="Q10">
-        <v>0.506</v>
-      </c>
-      <c r="R10">
-        <v>0.869</v>
-      </c>
-      <c r="S10">
-        <v>22.5</v>
-      </c>
-      <c r="T10">
-        <v>14.3</v>
-      </c>
-      <c r="U10">
-        <v>33.2</v>
-      </c>
-      <c r="V10">
-        <v>48.7</v>
-      </c>
-      <c r="W10">
-        <v>37.5</v>
-      </c>
-      <c r="X10" t="s">
-        <v>66</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z10" t="s">
-        <v>68</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>60</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>66</v>
-      </c>
-      <c r="AC10" t="s">
         <v>69</v>
-      </c>
-      <c r="AD10">
-        <v>428</v>
-      </c>
-      <c r="AE10">
-        <v>8</v>
-      </c>
-      <c r="AF10">
-        <v>0.286</v>
-      </c>
-      <c r="AG10">
-        <v>0.332</v>
-      </c>
-      <c r="AH10">
-        <v>1.9</v>
-      </c>
-      <c r="AI10">
-        <v>0.158</v>
-      </c>
-      <c r="AJ10">
-        <v>0.444</v>
-      </c>
-      <c r="AK10">
-        <v>24.3</v>
-      </c>
-      <c r="AL10">
-        <v>5.1</v>
-      </c>
-      <c r="AM10">
-        <v>2.82</v>
-      </c>
-      <c r="AN10">
-        <v>53.4</v>
-      </c>
-      <c r="AO10">
-        <v>24.3</v>
-      </c>
-      <c r="AP10">
-        <v>11.3</v>
-      </c>
-      <c r="AQ10">
-        <v>27.4</v>
-      </c>
-      <c r="AR10">
-        <v>1</v>
-      </c>
-      <c r="AS10">
-        <v>1</v>
-      </c>
-      <c r="AT10">
-        <v>0</v>
-      </c>
-      <c r="AU10">
-        <v>0</v>
-      </c>
-      <c r="AV10">
-        <v>1</v>
-      </c>
-      <c r="AW10">
-        <v>0</v>
-      </c>
-      <c r="AX10">
-        <v>1</v>
-      </c>
-      <c r="AY10" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>